<commit_message>
Version 4.0 全行程Track方式 Build 20260724-13
</commit_message>
<xml_diff>
--- a/data/travel_plans.xlsx
+++ b/data/travel_plans.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旅行計画" sheetId="1" r:id="Rf008b65fa5c04eec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旅行計画" sheetId="1" r:id="Re2193c11c5a247f3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,29 +13,25 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="4">
+  <x:fonts count="3">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
-      <x:sz val="16"/>
+      <x:sz val="14"/>
       <x:color rgb="FFFFFFFF"/>
-      <x:name val="Carlito"/>
-    </x:font>
-    <x:font>
-      <x:sz val="11"/>
-      <x:color rgb="FF1E3A8A"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
+      <x:color rgb="FF1E3A8A"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -49,12 +45,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFEFF6FF"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFDCE6F1"/>
+        <x:fgColor rgb="FFDBEAFE"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -65,7 +56,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="27">
+  <x:cellXfs count="22">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -84,40 +75,33 @@
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -283,10 +267,11 @@
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="36" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="38" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="38" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="34" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="36" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="48" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -304,99 +289,107 @@
       <x:c r="J1" s="5"/>
       <x:c r="K1" s="5"/>
       <x:c r="L1" s="5"/>
+      <x:c r="M1" s="5"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="12" t="str">
-        <x:v>Version 4.0 プラン連携テスト用。4行目の見出しは変更しないでください。</x:v>
-      </x:c>
-      <x:c r="B2" s="12"/>
-      <x:c r="C2" s="12"/>
-      <x:c r="D2" s="12"/>
-      <x:c r="E2" s="12"/>
-      <x:c r="F2" s="12"/>
-      <x:c r="G2" s="12"/>
-      <x:c r="H2" s="12"/>
-      <x:c r="I2" s="12"/>
-      <x:c r="J2" s="12"/>
-      <x:c r="K2" s="12"/>
-      <x:c r="L2" s="12"/>
+      <x:c r="A2" s="10" t="str">
+        <x:v>Version 4.0：全行程ルートはAIが作成する道路列。始点から終点までを連続Track GPXとして出力する。</x:v>
+      </x:c>
+      <x:c r="B2" s="10"/>
+      <x:c r="C2" s="10"/>
+      <x:c r="D2" s="10"/>
+      <x:c r="E2" s="10"/>
+      <x:c r="F2" s="10"/>
+      <x:c r="G2" s="10"/>
+      <x:c r="H2" s="10"/>
+      <x:c r="I2" s="10"/>
+      <x:c r="J2" s="10"/>
+      <x:c r="K2" s="10"/>
+      <x:c r="L2" s="10"/>
+      <x:c r="M2" s="10"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="20" t="str">
+      <x:c r="A4" s="16" t="str">
         <x:v>計画名</x:v>
       </x:c>
-      <x:c r="B4" s="20" t="str">
+      <x:c r="B4" s="16" t="str">
         <x:v>対象路線</x:v>
       </x:c>
-      <x:c r="C4" s="20" t="str">
+      <x:c r="C4" s="16" t="str">
         <x:v>始点</x:v>
       </x:c>
-      <x:c r="D4" s="20" t="str">
+      <x:c r="D4" s="16" t="str">
         <x:v>終点</x:v>
       </x:c>
-      <x:c r="E4" s="20" t="str">
+      <x:c r="E4" s="16" t="str">
         <x:v>距離(km)</x:v>
       </x:c>
-      <x:c r="F4" s="20" t="str">
+      <x:c r="F4" s="16" t="str">
         <x:v>所要時間</x:v>
       </x:c>
-      <x:c r="G4" s="20" t="str">
+      <x:c r="G4" s="16" t="str">
         <x:v>宿泊</x:v>
       </x:c>
-      <x:c r="H4" s="20" t="str">
+      <x:c r="H4" s="16" t="str">
         <x:v>優先度</x:v>
       </x:c>
-      <x:c r="I4" s="20" t="str">
+      <x:c r="I4" s="16" t="str">
         <x:v>季節</x:v>
       </x:c>
-      <x:c r="J4" s="20" t="str">
+      <x:c r="J4" s="16" t="str">
         <x:v>メモ</x:v>
       </x:c>
-      <x:c r="K4" s="20" t="str">
+      <x:c r="K4" s="16" t="str">
         <x:v>経由地</x:v>
       </x:c>
-      <x:c r="L4" s="20" t="str">
+      <x:c r="L4" s="16" t="str">
+        <x:v>全行程ルート</x:v>
+      </x:c>
+      <x:c r="M4" s="16" t="str">
         <x:v>GoogleマップURL</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="26" t="str">
+      <x:c r="A5" s="10" t="str">
         <x:v>7/12実走再現テスト</x:v>
       </x:c>
-      <x:c r="B5" s="26" t="str">
+      <x:c r="B5" s="10" t="str">
         <x:v>40→12→233→275→451→231</x:v>
       </x:c>
-      <x:c r="C5" s="26" t="str">
+      <x:c r="C5" s="10" t="str">
         <x:v>士別市</x:v>
       </x:c>
-      <x:c r="D5" s="26" t="str">
+      <x:c r="D5" s="10" t="str">
         <x:v>士別市</x:v>
       </x:c>
-      <x:c r="E5" s="26" t="n">
+      <x:c r="E5" s="10" t="n">
         <x:v>385.9</x:v>
       </x:c>
-      <x:c r="F5" s="26" t="str"/>
-      <x:c r="G5" s="26" t="str">
+      <x:c r="F5" s="10" t="str"/>
+      <x:c r="G5" s="10" t="str">
         <x:v>日帰り</x:v>
       </x:c>
-      <x:c r="H5" s="26" t="str">
+      <x:c r="H5" s="10" t="str">
         <x:v>テスト</x:v>
       </x:c>
-      <x:c r="I5" s="26" t="str">
+      <x:c r="I5" s="10" t="str">
         <x:v>夏</x:v>
       </x:c>
-      <x:c r="J5" s="26" t="str">
-        <x:v>Version 4.0のプラン連携確認用。7/12実走済みデータと同じ6路線を使用。</x:v>
-      </x:c>
-      <x:c r="K5" s="26" t="str">
+      <x:c r="J5" s="10" t="str">
+        <x:v>Version 4.0 全行程Track方式の検証用。7/12実走済みルートを始点から終点まで再現する。</x:v>
+      </x:c>
+      <x:c r="K5" s="10" t="str">
         <x:v>深川市→沼田町→雨竜町→滝川市→留萌市→増毛町</x:v>
       </x:c>
-      <x:c r="L5" s="26" t="str"/>
+      <x:c r="L5" s="10" t="str">
+        <x:v>40:旭川市→12:深川市→233:沼田町→275:滝川市→451:石狩市浜益区→231:留萌市→233:深川市→12:旭川市→40:士別市</x:v>
+      </x:c>
+      <x:c r="M5" s="10" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:L1"/>
-    <x:mergeCell ref="A2:L2"/>
+    <x:mergeCell ref="A1:M1"/>
+    <x:mergeCell ref="A2:M2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>